<commit_message>
Add operadora v2 audit outputs
</commit_message>
<xml_diff>
--- a/utils/insumos/regras_operadora.xlsx
+++ b/utils/insumos/regras_operadora.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -47,7 +44,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -55,22 +52,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -147,40 +135,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela_regras_operadora" displayName="Tabela_regras_operadora" ref="A1:N421" headerRowCount="1">
-  <autoFilter ref="A1:N421"/>
-  <tableColumns count="14">
-    <tableColumn id="1" name="OPERADORA"/>
-    <tableColumn id="2" name="APLICAR_SOMENTE_VAZIO"/>
-    <tableColumn id="3" name="COLUNA_FILTRO_1"/>
-    <tableColumn id="4" name="COMPARADOR_1"/>
-    <tableColumn id="5" name="VALOR_1"/>
-    <tableColumn id="6" name="COLUNA_FILTRO_2"/>
-    <tableColumn id="7" name="COMPARADOR_2"/>
-    <tableColumn id="8" name="VALOR_2"/>
-    <tableColumn id="9" name="COLUNA_FILTRO_3"/>
-    <tableColumn id="10" name="COMPARADOR_3"/>
-    <tableColumn id="11" name="VALOR_3"/>
-    <tableColumn id="12" name="ORDEM"/>
-    <tableColumn id="13" name="STATUS_ATIVO"/>
-    <tableColumn id="14" name="DESCRICAO"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela_comparadores" displayName="Tabela_comparadores" ref="A1:B7" headerRowCount="1">
-  <autoFilter ref="A1:B7"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="COMPARADOR"/>
-    <tableColumn id="2" name="DESCRICAO"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -479,7 +433,7 @@
     <col width="23" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
@@ -488,76 +442,76 @@
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="42" customWidth="1" min="14" max="14"/>
+    <col width="44" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>OPERADORA</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>APLICAR_SOMENTE_VAZIO</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>COLUNA_FILTRO_1</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>COMPARADOR_1</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>VALOR_1</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>COLUNA_FILTRO_2</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>COMPARADOR_2</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>VALOR_2</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>COLUNA_FILTRO_3</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>COMPARADOR_3</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>VALOR_3</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>ORDEM</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>STATUS_ATIVO</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>DESCRICAO</t>
         </is>
@@ -669,6 +623,21 @@
           <t>PR</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>CONTRATACAO</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>igual</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>rede propria</t>
+        </is>
+      </c>
       <c r="L4" t="n">
         <v>3</v>
       </c>
@@ -709,6 +678,21 @@
           <t>RS</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>CONTRATACAO</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>igual</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>rede propria</t>
+        </is>
+      </c>
       <c r="L5" t="n">
         <v>4</v>
       </c>
@@ -749,6 +733,21 @@
           <t>MG</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>CONTRATACAO</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>igual</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>rede propria</t>
+        </is>
+      </c>
       <c r="L6" t="n">
         <v>5</v>
       </c>
@@ -17515,9 +17514,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -17531,16 +17527,16 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>COMPARADOR</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>DESCRICAO</t>
         </is>
@@ -17620,8 +17616,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>